<commit_message>
Update campeggi.xlsx with new data
</commit_message>
<xml_diff>
--- a/campeggi.xlsx
+++ b/campeggi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Scattolin Marco\repos\PERSONAL_REPOS\france_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EA721C8-BC82-4D5F-BA4E-3D8A195E2C3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABBBF587-9BBE-4450-9562-F36C80F29A19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{88853F70-AB9D-42CD-ADB2-C63A4B0D3589}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="33">
   <si>
     <t xml:space="preserve"> Aire de la Ferme Froide</t>
   </si>
@@ -86,9 +86,6 @@
     <t>SI</t>
   </si>
   <si>
-    <t>??</t>
-  </si>
-  <si>
     <t>inviata mail richiesta per tutti e 4</t>
   </si>
   <si>
@@ -132,6 +129,12 @@
   </si>
   <si>
     <t>BAGNI</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>?</t>
   </si>
 </sst>
 </file>
@@ -139,10 +142,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
-    <numFmt numFmtId="166" formatCode="#,##0.00\ &quot;€&quot;"/>
+    <numFmt numFmtId="167" formatCode="ddd\ dd\ mmm\ yyyy"/>
+    <numFmt numFmtId="168" formatCode="\€\ #,##0.00;\€\ \(#,##0.00\);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -173,15 +176,34 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF1F2937"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F2937"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF1F4E78"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -190,18 +212,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
+        <fgColor rgb="FF1F4E78"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="1"/>
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAF2F8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -211,16 +239,175 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color rgb="FFD0D7DE"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color rgb="FFD0D7DE"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color rgb="FFD0D7DE"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color rgb="FFD0D7DE"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7DE"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7DE"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1F4E78"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F4E78"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7DE"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7DE"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D7DE"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F4E78"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1F4E78"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7DE"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1F4E78"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F4E78"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1F4E78"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7DE"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D7DE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D7DE"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1F4E78"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7DE"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D7DE"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F4E78"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7DE"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1F4E78"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D7DE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D7DE"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7DE"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1F4E78"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D7DE"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F4E78"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1F4E78"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7DE"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD0D7DE"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7DE"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7DE"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD0D7DE"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7DE"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1F4E78"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD0D7DE"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7DE"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1F4E78"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1F4E78"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F4E78"/>
       </bottom>
       <diagonal/>
     </border>
@@ -229,7 +416,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -237,44 +424,104 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -609,265 +856,289 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="525" row="7">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{EC0CCFCE-A7C2-46B5-9F4A-CF2A4B78BD9A}">
+  <we:reference id="29673e3c-d826-4f00-92ee-162334a52b1a" version="1.0.0.8" store="EXCatalog" storeType="EXCatalog"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;f25e0379-bddb-44d4-82a0-7d232a8d4ee2&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F992FBED-BBE0-49C8-B2A8-2CE7A077F8A5}">
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultColWidth="110.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.7265625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="16.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="81.1796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.26953125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="21.7265625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="11.453125" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="110.81640625" style="3"/>
+    <col min="1" max="1" width="6.90625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="27.26953125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="30.90625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="41.81640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="40" style="1" customWidth="1"/>
+    <col min="6" max="6" width="23.6328125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="20" style="1" customWidth="1"/>
+    <col min="8" max="8" width="12.7265625" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="110.81640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="15" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:8" s="3" customFormat="1" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="F1" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="12" t="s">
+      <c r="G1" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="H1" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="H1" s="12" t="s">
+    </row>
+    <row r="2" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="16">
+        <v>1</v>
+      </c>
+      <c r="B2" s="17">
+        <v>46255</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="27" t="s">
         <v>31</v>
       </c>
+      <c r="G2" s="18"/>
+      <c r="H2" s="19"/>
     </row>
-    <row r="2" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="4">
-        <v>1</v>
-      </c>
-      <c r="B2" s="10">
-        <v>46255</v>
-      </c>
-      <c r="C2" s="4" t="s">
+    <row r="3" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="11">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6">
+        <v>46256</v>
+      </c>
+      <c r="C3" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D3" s="28"/>
+      <c r="E3" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="7"/>
+      <c r="H3" s="14"/>
+    </row>
+    <row r="4" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="10">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4">
+        <v>46257</v>
+      </c>
+      <c r="C4" s="30" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="30"/>
+      <c r="E4" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="31" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="5"/>
+      <c r="H4" s="13"/>
+    </row>
+    <row r="5" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="11">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6">
+        <v>46258</v>
+      </c>
+      <c r="C5" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="7">
+        <v>11</v>
+      </c>
+      <c r="H5" s="14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="10">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4">
+        <v>46259</v>
+      </c>
+      <c r="C6" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="E6" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="31" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="5">
         <v>25</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F2" s="6"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="4"/>
+      <c r="H6" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" s="7">
-        <v>2</v>
-      </c>
-      <c r="B3" s="11">
-        <v>46256</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="7"/>
-      <c r="E3" s="8" t="s">
+    <row r="7" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="11">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6">
+        <v>46260</v>
+      </c>
+      <c r="C7" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="28" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="29" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="10">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4">
+        <v>46261</v>
+      </c>
+      <c r="C8" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="31" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" s="5">
+        <v>51</v>
+      </c>
+      <c r="H8" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="11">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6">
+        <v>46262</v>
+      </c>
+      <c r="C9" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" s="14"/>
-      <c r="H3" s="7"/>
+      <c r="D9" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="23"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="14"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" s="7">
-        <v>3</v>
-      </c>
-      <c r="B4" s="11">
-        <v>46257</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="14"/>
-      <c r="H4" s="7"/>
+    <row r="10" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4">
+        <v>46263</v>
+      </c>
+      <c r="C10" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="24"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="13"/>
     </row>
-    <row r="5" spans="1:8" ht="87" x14ac:dyDescent="0.35">
-      <c r="A5" s="7">
-        <v>4</v>
-      </c>
-      <c r="B5" s="11">
-        <v>46258</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="14">
-        <v>11</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" s="7">
-        <v>5</v>
-      </c>
-      <c r="B6" s="11">
-        <v>46259</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" s="14">
+    <row r="11" spans="1:8" ht="22" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="12">
+        <v>10</v>
+      </c>
+      <c r="B11" s="8">
+        <v>46264</v>
+      </c>
+      <c r="C11" s="32" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="H6" s="7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="4">
-        <v>6</v>
-      </c>
-      <c r="B7" s="10">
-        <v>46260</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="G7" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="58" x14ac:dyDescent="0.35">
-      <c r="A8" s="7">
-        <v>7</v>
-      </c>
-      <c r="B8" s="11">
-        <v>46261</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" s="14">
-        <v>51</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" s="4">
-        <v>8</v>
-      </c>
-      <c r="B9" s="10">
-        <v>46262</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E9" s="4"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="4"/>
-    </row>
-    <row r="10" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A10" s="4">
-        <v>9</v>
-      </c>
-      <c r="B10" s="10">
-        <v>46263</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="4"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="4"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" s="4">
-        <v>10</v>
-      </c>
-      <c r="B11" s="10">
-        <v>46264</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11" s="4"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="4"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="33"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="15"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
Sync confirmed campsites from campeggi.xlsx to itinerary
Update day cards in index.html to reflect the latest confirmed
campsites in campeggi.xlsx (source of truth): Camping Mont Blanc Plage
(G1), Camping de la Cité d'Aleth (G6), Camping Le Moulin Fort (G8-G9),
and Camping Ferrand replacing the previous Aix-les-Bains placeholder
(G10, still to confirm).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/campeggi.xlsx
+++ b/campeggi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Scattolin Marco\repos\PERSONAL_REPOS\france_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABBBF587-9BBE-4450-9562-F36C80F29A19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03FBE5E4-4D0B-4261-9DD9-5EC7F7110373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{88853F70-AB9D-42CD-ADB2-C63A4B0D3589}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="38">
   <si>
     <t xml:space="preserve"> Aire de la Ferme Froide</t>
   </si>
@@ -62,9 +62,6 @@
     <t>Saint Malò</t>
   </si>
   <si>
-    <t>Camping Les Ilots</t>
-  </si>
-  <si>
     <t>Phare de Mean Ruz</t>
   </si>
   <si>
@@ -74,9 +71,6 @@
     <t>https://www.pitchup.com/it/campsites/france/bretagne/cotes-darmor/trelevern/camping_port_lepine/?arrive=2026-08-27&amp;depart=2026-08-28&amp;type=10&amp;adults=2&amp;child_ages=15%2C17&amp;children=2&amp;gclsrc=aw.ds&amp;gbraid=0AAAAAD0B4Qwiu-PsUNZulWDW4LKzm1O0j</t>
   </si>
   <si>
-    <t>https://www.camperonline.it/sosta-camper/aree-di-sosta/francia/aire-de-campingcars-les-ilots/11597</t>
-  </si>
-  <si>
     <t>https://www.pitchup.com/it/campsites/france/basse-normandie/calvados/juaye-mondaye/aire-de-la-ferme-froide/?utm_source=google&amp;utm_source_platform=Google+Ads&amp;utm_medium=cpc&amp;utm_campaign=_French_Areas_France__None_%7C_None__DSAFeed&amp;utm_campaignid=23807923187&amp;ads_rl=9159830176&amp;&amp;&amp;&amp;gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=23807923187&amp;gbraid=0AAAAAD0B4QxBJVD4I-1n0o3lvDM16mIHz</t>
   </si>
   <si>
@@ -86,9 +80,6 @@
     <t>SI</t>
   </si>
   <si>
-    <t>inviata mail richiesta per tutti e 4</t>
-  </si>
-  <si>
     <t>Chamonix</t>
   </si>
   <si>
@@ -113,9 +104,6 @@
     <t>Camping Mont Blanc Plage</t>
   </si>
   <si>
-    <t>TBD</t>
-  </si>
-  <si>
     <t>LINK</t>
   </si>
   <si>
@@ -135,6 +123,33 @@
   </si>
   <si>
     <t>?</t>
+  </si>
+  <si>
+    <t>NOTE</t>
+  </si>
+  <si>
+    <t>Il sito segnalava arrivo massimo ore 19 - chiamare per conferma ingresso anche entro le 21 - +33450581428 oppure +33450581204</t>
+  </si>
+  <si>
+    <t>https://premium-camplive.com/fr/campingdelacitedaleth/</t>
+  </si>
+  <si>
+    <t>City Kamp</t>
+  </si>
+  <si>
+    <t>Camping de la Cité d'Aleth</t>
+  </si>
+  <si>
+    <t>https://www.pitchup.com/it/campsites/france/centre/indre-et-loire/francueil/camping-le-moulin-fort/</t>
+  </si>
+  <si>
+    <t>Camping Le Moulin Fort</t>
+  </si>
+  <si>
+    <t>https://www.pitchup.com/it/campsites/france/rhone-alpes/savoie/lepin-le-lac/camping-ferrand/</t>
+  </si>
+  <si>
+    <t>Camping Ferrand</t>
   </si>
 </sst>
 </file>
@@ -142,8 +157,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="167" formatCode="ddd\ dd\ mmm\ yyyy"/>
-    <numFmt numFmtId="168" formatCode="\€\ #,##0.00;\€\ \(#,##0.00\);&quot;-&quot;"/>
+    <numFmt numFmtId="164" formatCode="ddd\ dd\ mmm\ yyyy"/>
+    <numFmt numFmtId="165" formatCode="\€\ #,##0.00;\€\ \(#,##0.00\);&quot;-&quot;"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -427,22 +442,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -466,10 +481,10 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -490,15 +505,9 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -521,6 +530,12 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -880,7 +895,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F992FBED-BBE0-49C8-B2A8-2CE7A077F8A5}">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultColWidth="110.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6.90625" style="1" customWidth="1"/>
@@ -890,11 +905,11 @@
     <col min="5" max="5" width="40" style="1" customWidth="1"/>
     <col min="6" max="6" width="23.6328125" style="2" customWidth="1"/>
     <col min="7" max="7" width="20" style="1" customWidth="1"/>
-    <col min="8" max="8" width="12.7265625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="6.6328125" style="2" customWidth="1"/>
     <col min="9" max="16384" width="110.81640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="3" customFormat="1" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:9" s="3" customFormat="1" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="20" t="s">
         <v>6</v>
       </c>
@@ -905,240 +920,263 @@
         <v>2</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E1" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="F1" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="G1" s="21" t="s">
+      <c r="I1" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="H1" s="22" t="s">
-        <v>30</v>
-      </c>
     </row>
-    <row r="2" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="16">
         <v>1</v>
       </c>
       <c r="B2" s="17">
         <v>46255</v>
       </c>
-      <c r="C2" s="26" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2" s="26" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="34" t="s">
-        <v>23</v>
-      </c>
-      <c r="F2" s="27" t="s">
-        <v>31</v>
+      <c r="C2" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="29" t="s">
+        <v>13</v>
       </c>
       <c r="G2" s="18"/>
-      <c r="H2" s="19"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="19" t="s">
+        <v>30</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="11">
         <v>2</v>
       </c>
       <c r="B3" s="6">
         <v>46256</v>
       </c>
-      <c r="C3" s="28" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="28"/>
+      <c r="C3" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="26" t="s">
+        <v>32</v>
+      </c>
       <c r="E3" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" s="29" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="F3" s="27" t="s">
+        <v>13</v>
       </c>
       <c r="G3" s="7"/>
-      <c r="H3" s="14"/>
+      <c r="H3" s="27"/>
+      <c r="I3" s="14"/>
     </row>
-    <row r="4" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="10">
         <v>3</v>
       </c>
       <c r="B4" s="4">
         <v>46257</v>
       </c>
-      <c r="C4" s="30" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="30"/>
+      <c r="C4" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="28" t="s">
+        <v>32</v>
+      </c>
       <c r="E4" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" s="31" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="F4" s="29" t="s">
+        <v>13</v>
       </c>
       <c r="G4" s="5"/>
-      <c r="H4" s="13"/>
+      <c r="H4" s="29"/>
+      <c r="I4" s="13"/>
     </row>
-    <row r="5" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="11">
         <v>4</v>
       </c>
       <c r="B5" s="6">
         <v>46258</v>
       </c>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="28" t="s">
+      <c r="D5" s="26" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="29" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="7">
-        <v>11</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>15</v>
+      <c r="G5" s="7"/>
+      <c r="H5" s="27"/>
+      <c r="I5" s="14" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="10">
         <v>5</v>
       </c>
       <c r="B6" s="4">
         <v>46259</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="35" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="31" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" s="5">
-        <v>25</v>
-      </c>
-      <c r="H6" s="13" t="s">
-        <v>15</v>
+      <c r="E6" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="5"/>
+      <c r="H6" s="29"/>
+      <c r="I6" s="13" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="11">
         <v>6</v>
       </c>
       <c r="B7" s="6">
         <v>46260</v>
       </c>
-      <c r="C7" s="28" t="s">
+      <c r="C7" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="29" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>32</v>
+      <c r="D7" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="7"/>
+      <c r="H7" s="27"/>
+      <c r="I7" s="14" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="10">
         <v>7</v>
       </c>
       <c r="B8" s="4">
         <v>46261</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="28" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="30" t="s">
+      <c r="E8" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="31" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" s="5">
-        <v>51</v>
-      </c>
-      <c r="H8" s="13" t="s">
-        <v>15</v>
+      <c r="F8" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="5"/>
+      <c r="H8" s="29"/>
+      <c r="I8" s="13" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="11">
         <v>8</v>
       </c>
       <c r="B9" s="6">
         <v>46262</v>
       </c>
-      <c r="C9" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="28" t="s">
-        <v>25</v>
-      </c>
-      <c r="E9" s="23"/>
-      <c r="F9" s="29"/>
+      <c r="C9" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" s="27" t="s">
+        <v>13</v>
+      </c>
       <c r="G9" s="7"/>
-      <c r="H9" s="14"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="14"/>
     </row>
-    <row r="10" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="10">
         <v>9</v>
       </c>
       <c r="B10" s="4">
         <v>46263</v>
       </c>
-      <c r="C10" s="30" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="30" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" s="24"/>
-      <c r="F10" s="31"/>
+      <c r="C10" s="28" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="E10" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="F10" s="29" t="s">
+        <v>13</v>
+      </c>
       <c r="G10" s="5"/>
-      <c r="H10" s="13"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="13"/>
     </row>
-    <row r="11" spans="1:8" ht="22" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:9" ht="22" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="12">
         <v>10</v>
       </c>
       <c r="B11" s="8">
         <v>46264</v>
       </c>
-      <c r="C11" s="32" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11" s="32" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11" s="25"/>
-      <c r="F11" s="33"/>
+      <c r="C11" s="30" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="E11" s="35" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" s="31" t="s">
+        <v>27</v>
+      </c>
       <c r="G11" s="9"/>
-      <c r="H11" s="15"/>
+      <c r="H11" s="31"/>
+      <c r="I11" s="15"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1148,6 +1186,9 @@
     <hyperlink ref="E7" r:id="rId3" xr:uid="{2BEE32A4-DCFA-4FD6-AB1A-4ED9A626A0A4}"/>
     <hyperlink ref="E8" r:id="rId4" xr:uid="{743CCEA3-A555-42CB-9007-C8BA23F1E637}"/>
     <hyperlink ref="E2" r:id="rId5" xr:uid="{AA7F2F17-402C-4E22-857F-DD6384A4CEB3}"/>
+    <hyperlink ref="E9" r:id="rId6" xr:uid="{9A834760-3113-403A-8BC4-136933E97C75}"/>
+    <hyperlink ref="E10" r:id="rId7" xr:uid="{CB1A6F40-1D26-41B1-999E-BD9ABAA92737}"/>
+    <hyperlink ref="E11" r:id="rId8" xr:uid="{42F18656-8446-4690-A670-2BE66AE1E4F0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update campeggi.xlsx with new campsite information
</commit_message>
<xml_diff>
--- a/campeggi.xlsx
+++ b/campeggi.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Scattolin Marco\repos\PERSONAL_REPOS\france_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03FBE5E4-4D0B-4261-9DD9-5EC7F7110373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03815C93-D990-4ECA-9FD7-4414C27D4B0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{88853F70-AB9D-42CD-ADB2-C63A4B0D3589}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="37">
   <si>
     <t xml:space="preserve"> Aire de la Ferme Froide</t>
   </si>
@@ -119,18 +119,12 @@
     <t>BAGNI</t>
   </si>
   <si>
-    <t>NO</t>
-  </si>
-  <si>
     <t>?</t>
   </si>
   <si>
     <t>NOTE</t>
   </si>
   <si>
-    <t>Il sito segnalava arrivo massimo ore 19 - chiamare per conferma ingresso anche entro le 21 - +33450581428 oppure +33450581204</t>
-  </si>
-  <si>
     <t>https://premium-camplive.com/fr/campingdelacitedaleth/</t>
   </si>
   <si>
@@ -150,6 +144,9 @@
   </si>
   <si>
     <t>Camping Ferrand</t>
+  </si>
+  <si>
+    <t>Info allo +33450581428 oppure +33450581204</t>
   </si>
 </sst>
 </file>
@@ -935,7 +932,7 @@
         <v>26</v>
       </c>
       <c r="I1" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -960,7 +957,7 @@
       <c r="G2" s="18"/>
       <c r="H2" s="29"/>
       <c r="I2" s="19" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -974,7 +971,7 @@
         <v>15</v>
       </c>
       <c r="D3" s="26" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E3" s="23" t="s">
         <v>16</v>
@@ -997,7 +994,7 @@
         <v>15</v>
       </c>
       <c r="D4" s="28" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E4" s="24" t="s">
         <v>16</v>
@@ -1070,10 +1067,10 @@
         <v>7</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E7" s="34" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F7" s="27" t="s">
         <v>13</v>
@@ -1081,7 +1078,7 @@
       <c r="G7" s="7"/>
       <c r="H7" s="27"/>
       <c r="I7" s="14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -1120,10 +1117,10 @@
         <v>17</v>
       </c>
       <c r="D9" s="26" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E9" s="34" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F9" s="27" t="s">
         <v>13</v>
@@ -1143,10 +1140,10 @@
         <v>19</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F10" s="29" t="s">
         <v>13</v>
@@ -1166,13 +1163,13 @@
         <v>18</v>
       </c>
       <c r="D11" s="30" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E11" s="35" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F11" s="31" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="G11" s="9"/>
       <c r="H11" s="31"/>

</xml_diff>